<commit_message>
docs: separate weapons, armor and jewelry with borders in heirlooms.xlsx
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NKhm7yXfn5QStARX3kAcsE
</commit_message>
<xml_diff>
--- a/docs/heirlooms.xlsx
+++ b/docs/heirlooms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Axel\projects\misc\archipelawow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Axel\projects\misc\archipelawow\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C889558-3DE7-473E-A961-5C6BA04228BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1DD78F-FC74-4152-8F5B-204E425182E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8326D24-0A60-47AA-B677-58249B967B9A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8326D24-0A60-47AA-B677-58249B967B9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -219,7 +219,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -227,17 +227,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -880,34 +892,34 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="2">
-        <v>1</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0</v>
-      </c>
-      <c r="I10" s="2">
-        <v>0</v>
-      </c>
-      <c r="J10" s="2">
+      <c r="C10" s="4">
+        <v>1</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4">
         <v>0</v>
       </c>
     </row>
@@ -1264,34 +1276,34 @@
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="2">
-        <v>1</v>
-      </c>
-      <c r="D22" s="2">
-        <v>1</v>
-      </c>
-      <c r="E22" s="2">
-        <v>1</v>
-      </c>
-      <c r="F22" s="2">
-        <v>1</v>
-      </c>
-      <c r="G22" s="2">
-        <v>1</v>
-      </c>
-      <c r="H22" s="2">
-        <v>1</v>
-      </c>
-      <c r="I22" s="2">
-        <v>0</v>
-      </c>
-      <c r="J22" s="2">
+      <c r="C22" s="4">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4">
+        <v>1</v>
+      </c>
+      <c r="E22" s="4">
+        <v>1</v>
+      </c>
+      <c r="F22" s="4">
+        <v>1</v>
+      </c>
+      <c r="G22" s="4">
+        <v>1</v>
+      </c>
+      <c r="H22" s="4">
+        <v>1</v>
+      </c>
+      <c r="I22" s="4">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>